<commit_message>
Giai đoạn 1 v1
</commit_message>
<xml_diff>
--- a/docs/schedule.xlsx
+++ b/docs/schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATN_NGUYEN_CHI_THANH\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C520CD13-E261-4597-9099-A94DDE8A137D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A46A5CB-BAA6-4868-961A-531FD91C265E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
     <t>Thiết kế UC, Database, API</t>
   </si>
   <si>
-    <t>23/09/2025</t>
+    <t>26/09/2025</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Bổ sung giai đoạn
</commit_message>
<xml_diff>
--- a/docs/schedule.xlsx
+++ b/docs/schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATN_NGUYEN_CHI_THANH\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A46A5CB-BAA6-4868-961A-531FD91C265E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD8580D2-815A-433D-8F81-7D7798FEBE72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Lịch trình công việc</t>
   </si>
@@ -52,6 +52,36 @@
   </si>
   <si>
     <t>26/09/2025</t>
+  </si>
+  <si>
+    <t>Giai đoạn 2</t>
+  </si>
+  <si>
+    <t>28/9/2025</t>
+  </si>
+  <si>
+    <t>Hoàn thành các API CRUD chính</t>
+  </si>
+  <si>
+    <t>Giai đoạn 3</t>
+  </si>
+  <si>
+    <t>20/10/2015</t>
+  </si>
+  <si>
+    <t>Xây dựng giao diện cho hệ thống</t>
+  </si>
+  <si>
+    <t>Giai đoạn 4</t>
+  </si>
+  <si>
+    <t>20/10/2025</t>
+  </si>
+  <si>
+    <t>31/10/2025</t>
+  </si>
+  <si>
+    <t>Ghép API vào giao diện</t>
   </si>
 </sst>
 </file>
@@ -111,12 +141,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -403,7 +434,7 @@
     <col min="1" max="1" width="17.1796875" customWidth="1"/>
     <col min="2" max="2" width="11.36328125" customWidth="1"/>
     <col min="3" max="3" width="10.7265625" customWidth="1"/>
-    <col min="4" max="4" width="23.54296875" customWidth="1"/>
+    <col min="4" max="4" width="28.36328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -443,22 +474,46 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
+      <c r="A4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="3">
+        <v>45940</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
+      <c r="A5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="3">
+        <v>45971</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
+      <c r="A6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="1"/>

</xml_diff>